<commit_message>
fix: show Tunisia fiscal stamp/withholding on default invoice template
Now that invoice PDF always follows the Excel template, pdf-tunisia.tsx
no longer renders for any organization. Without this, an org using
fiscalStampEnabled/withholdingTaxEnabled but no custom uploaded
template would silently lose those fields from their printed invoice.

Also updates CLAUDE.md's xlsx_export.go, layouts.ts, details.tsx, and
Tunisia-support entries, which still described the pre-unification
architecture (marker locked to column A, invoiceLayout selecting a
React-PDF component, PDFPreview still present).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014RJ1QcRJZ9C1WCAVsFGeRw
</commit_message>
<xml_diff>
--- a/db/templates/invoice_default.xlsx
+++ b/db/templates/invoice_default.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
   <si>
     <t>{{organization.name}}</t>
   </si>
@@ -117,6 +117,12 @@
   </si>
   <si>
     <t>IBAN: {{organization.iban}} | Bank: {{organization.bankName}}</t>
+  </si>
+  <si>
+    <t>Fiscal stamp: {{invoice.fiscalStampAmount}}</t>
+  </si>
+  <si>
+    <t>Withholding tax ({{invoice.withholdingTaxRate}}): {{invoice.withholdingTaxAmount}}</t>
   </si>
   <si>
     <t>Available template placeholders</t>
@@ -833,6 +839,16 @@
         <v>33</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>35</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A13:B13"/>
@@ -852,20 +868,20 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>15</v>
@@ -873,47 +889,47 @@
     </row>
     <row r="5">
       <c r="A5" s="7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11">
@@ -921,71 +937,71 @@
         <v>0</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12">
       <c r="B12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C13" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C14" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C16" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C17" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C18" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C19" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20">
@@ -993,68 +1009,68 @@
         <v>11</v>
       </c>
       <c r="C20" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C23" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C25" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C26" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C27" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="29">
@@ -1062,7 +1078,7 @@
         <v>25</v>
       </c>
       <c r="C29" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30">
@@ -1070,7 +1086,7 @@
         <v>20</v>
       </c>
       <c r="C30" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="31">
@@ -1086,7 +1102,7 @@
         <v>22</v>
       </c>
       <c r="C32" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="33">
@@ -1094,7 +1110,7 @@
         <v>23</v>
       </c>
       <c r="C33" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
     </row>
     <row r="34">
@@ -1102,12 +1118,12 @@
         <v>24</v>
       </c>
       <c r="C34" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="7" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="36">
@@ -1115,7 +1131,7 @@
         <v>27</v>
       </c>
       <c r="C36" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="37">
@@ -1123,7 +1139,7 @@
         <v>29</v>
       </c>
       <c r="C37" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="38">
@@ -1131,55 +1147,55 @@
         <v>31</v>
       </c>
       <c r="C38" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="39">
       <c r="B39" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C39" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="40">
       <c r="B40" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C40" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="41">
       <c r="B41" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C41" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C42" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C43" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
     </row>
     <row r="44">
       <c r="B44" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C44" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: fit invoice Excel template to one page wide for PDF export
Verified end-to-end for the first time by building the real Docker
image, running the container, and converting a live invoice to PDF via
LibreOffice: with no page setup at all, the six-column line-item table
didn't fit the default paper width, silently splitting every invoice
across two PDF pages (A-B on page 1, C-F on page 2) even though the
header/data alignment fix earlier this session was otherwise correct.
Excel itself shows no sign of this since it isn't paginated there.

FitToWidth=1/FitToHeight=0 (via SetSheetProps's FitToPage plus
SetPageLayout) scales the sheet to always fit one page wide while
leaving height unconstrained, so a long line-item list still
paginates vertically instead of being squeezed onto one page.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014RJ1QcRJZ9C1WCAVsFGeRw
</commit_message>
<xml_diff>
--- a/db/templates/invoice_default.xlsx
+++ b/db/templates/invoice_default.xlsx
@@ -694,6 +694,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -854,6 +857,7 @@
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A14:B14"/>
   </mergeCells>
+  <pageSetup fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fix: blank the withholding-tax line entirely when unset on invoice PDFs
The embedded invoice template built "Withholding tax ({{rate}}): {{amount}}"
as static text around two nullable placeholders. Every organization that
doesn't use Tunisia's opt-in withholding-tax feature — virtually all of
them — has both fields nil, so this rendered as a broken-looking
"Withholding tax (): " on every single invoice PDF this app has ever
exported (found by actually exporting a real invoice to PDF and reading
it, not just opening the .xlsx).

Replaces the two placeholders with one Go-computed invoice.withholdingTaxLine
that's either the fully-formatted line or entirely blank, same pattern
every other computed value on this template already follows. Regenerated
the embedded default via db/templates/gen (only invoice_default.xlsx
changes — withholding tax is invoice-only).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GftgB3L1qg1JAibuMakA2G
</commit_message>
<xml_diff>
--- a/db/templates/invoice_default.xlsx
+++ b/db/templates/invoice_default.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
   <si>
     <t>{{organization.name}}</t>
   </si>
@@ -125,7 +125,7 @@
     <t>Fiscal stamp: {{invoice.fiscalStampAmount}}</t>
   </si>
   <si>
-    <t>Withholding tax ({{invoice.withholdingTaxRate}}): {{invoice.withholdingTaxAmount}}</t>
+    <t>{{invoice.withholdingTaxLine}}</t>
   </si>
   <si>
     <t>Available template placeholders</t>
@@ -311,16 +311,7 @@
     <t>Tunisia timbre fiscal — flat duty, formatted with currency (0 if unused)</t>
   </si>
   <si>
-    <t>{{invoice.withholdingTaxRate}}</t>
-  </si>
-  <si>
-    <t>Withholding tax rate percentage, blank if unset</t>
-  </si>
-  <si>
-    <t>{{invoice.withholdingTaxAmount}}</t>
-  </si>
-  <si>
-    <t>Withholding tax amount, formatted with currency, blank if unset</t>
+    <t>Full "Withholding tax (12%): 40.00 EUR" line, entirely blank (not just the rate/amount) if unset</t>
   </si>
   <si>
     <t>{{organization.iban}}</t>
@@ -1200,63 +1191,55 @@
     </row>
     <row r="41">
       <c r="B41" t="s">
+        <v>35</v>
+      </c>
+      <c r="C41" t="s">
         <v>97</v>
-      </c>
-      <c r="C41" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="s">
+        <v>98</v>
+      </c>
+      <c r="C42" t="s">
         <v>99</v>
-      </c>
-      <c r="C42" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="s">
+        <v>100</v>
+      </c>
+      <c r="C43" t="s">
         <v>101</v>
       </c>
-      <c r="C43" t="s">
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" t="s">
+    <row r="45">
+      <c r="B45" t="s">
         <v>103</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C45" t="s">
         <v>104</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="7" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="46">
       <c r="B46" t="s">
+        <v>105</v>
+      </c>
+      <c r="C46" t="s">
         <v>106</v>
-      </c>
-      <c r="C46" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="47">
       <c r="B47" t="s">
+        <v>107</v>
+      </c>
+      <c r="C47" t="s">
         <v>108</v>
-      </c>
-      <c r="C47" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="B48" t="s">
-        <v>110</v>
-      </c>
-      <c r="C48" t="s">
-        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -1265,7 +1248,7 @@
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A28:C28"/>
     <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A44:C44"/>
   </mergeCells>
 </worksheet>
 </file>
</xml_diff>